<commit_message>
Fix malformed sheet1.xml in vegetation data-entry template
The permanence_class validation list contained "Ephemeral < 7 days";
openxlsx wrote the raw "<" into the x14:formula1 element without
escaping it, which Excel's parser rejected as an illegal qualified
name character. The whole plots sheet then failed to load.

Drop permanence_class from the Excel template altogether, matching
the recent removal from the PDF field form — water permanence is
derived from NDWI / LiDAR imagery in analysis/water/, not recorded
at the plot.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/templates/vegetation_hydrology_data_entry.xlsx
+++ b/inst/templates/vegetation_hydrology_data_entry.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
   <si>
     <t xml:space="preserve">project_id</t>
   </si>
@@ -106,9 +106,6 @@
     <t xml:space="preserve">ind_frost_hummocks</t>
   </si>
   <si>
-    <t xml:space="preserve">permanence_class</t>
-  </si>
-  <si>
     <t xml:space="preserve">determination</t>
   </si>
   <si>
@@ -190,9 +187,6 @@
     <t xml:space="preserve">FALSE</t>
   </si>
   <si>
-    <t xml:space="preserve">Semi-permanent</t>
-  </si>
-  <si>
     <t xml:space="preserve">Wetland</t>
   </si>
   <si>
@@ -274,7 +268,7 @@
     <t xml:space="preserve">plots — columns</t>
   </si>
   <si>
-    <t xml:space="preserve">plot_id: primary key (must match species sheet) | date: YYYY-MM-DD | datum: NAD83 or WGS84 | outlet: None / Surface / Subsurface / Both | hydro_ph / hydro_ec (uS/cm) / hydro_ppm (TDS) / hydro_temp (degC): in-situ multi-probe readings, leave blank if not measured | ind_*: TRUE if indicator was observed, FALSE if not (11 indicator columns) | permanence_class (per GWPWB): Ephemeral &lt;7d / Temporary (1-4 wk) / Seasonal (5-17 wk) / Semi-Permanent (18-40 wk) / Intermittent (41-51 wk) / Permanent (52 wk) | determination: Wetland / Non-wetland / Inconclusive | dom_criterion: Met / Not met / Marginal | remarks: combined hydrology notes and general observations</t>
+    <t xml:space="preserve">plot_id: primary key (must match species sheet) | date: YYYY-MM-DD | datum: NAD83 or WGS84 | outlet: None / Surface / Subsurface / Both | hydro_ph / hydro_ec (uS/cm) / hydro_ppm (TDS) / hydro_temp (degC): in-situ multi-probe readings, leave blank if not measured | ind_*: TRUE if indicator was observed, FALSE if not (11 indicator columns) | determination: Wetland / Non-wetland / Inconclusive | dom_criterion: Met / Not met / Marginal | remarks: combined hydrology notes and general observations</t>
   </si>
   <si>
     <t xml:space="preserve">species — columns</t>
@@ -672,7 +666,429 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?><worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac xr xr2 xr3" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3"> <sheetPr><tabColor rgb="FF2E5090"/></sheetPr> <dimension ref="A1"/> <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/> <cols><col min="1" max="1" width="14.71" hidden="0" customWidth="1"/><col min="2" max="2" width="12.71" hidden="0" customWidth="1"/><col min="3" max="3" width="12.71" hidden="0" customWidth="1"/><col min="4" max="4" width="16.71" hidden="0" customWidth="1"/><col min="5" max="5" width="12.71" hidden="0" customWidth="1"/><col min="6" max="6" width="12.71" hidden="0" customWidth="1"/><col min="7" max="7" width="12.71" hidden="0" customWidth="1"/><col min="8" max="8" width="9.71" hidden="0" customWidth="1"/><col min="9" max="9" width="22.71" hidden="0" customWidth="1"/><col min="10" max="10" width="9.71" hidden="0" customWidth="1"/><col min="11" max="11" width="12.71" hidden="0" customWidth="1"/><col min="12" max="12" width="16.71" hidden="0" customWidth="1"/><col min="13" max="13" width="10.71" hidden="0" customWidth="1"/><col min="14" max="14" width="10.71" hidden="0" customWidth="1"/><col min="15" max="15" width="12.71" hidden="0" customWidth="1"/><col min="16" max="16" width="7.71" hidden="0" customWidth="1"/><col min="17" max="17" width="8.71" hidden="0" customWidth="1"/><col min="18" max="18" width="8.71" hidden="0" customWidth="1"/><col min="19" max="19" width="8.71" hidden="0" customWidth="1"/><col min="20" max="20" width="10.71" hidden="0" customWidth="1"/><col min="21" max="21" width="10.71" hidden="0" customWidth="1"/><col min="22" max="22" width="10.71" hidden="0" customWidth="1"/><col min="23" max="23" width="10.71" hidden="0" customWidth="1"/><col min="24" max="24" width="10.71" hidden="0" customWidth="1"/><col min="25" max="25" width="10.71" hidden="0" customWidth="1"/><col min="26" max="26" width="10.71" hidden="0" customWidth="1"/><col min="27" max="27" width="10.71" hidden="0" customWidth="1"/><col min="28" max="28" width="10.71" hidden="0" customWidth="1"/><col min="29" max="29" width="10.71" hidden="0" customWidth="1"/><col min="30" max="30" width="10.71" hidden="0" customWidth="1"/><col min="31" max="31" width="16.71" hidden="0" customWidth="1"/><col min="32" max="32" width="13.71" hidden="0" customWidth="1"/><col min="33" max="33" width="11.71" hidden="0" customWidth="1"/><col min="34" max="34" width="10.71" hidden="0" customWidth="1"/><col min="35" max="35" width="10.71" hidden="0" customWidth="1"/><col min="36" max="36" width="10.71" hidden="0" customWidth="1"/><col min="37" max="37" width="9.71" hidden="0" customWidth="1"/><col min="38" max="38" width="9.71" hidden="0" customWidth="1"/><col min="39" max="39" width="40.71" hidden="0" customWidth="1"/></cols><sheetData><row r="1" ht="38" customHeight="1"><c r="A1" s="1" t="s"><v>0</v></c><c r="B1" s="1" t="s"><v>1</v></c><c r="C1" s="1" t="s"><v>2</v></c><c r="D1" s="1" t="s"><v>3</v></c><c r="E1" s="1" t="s"><v>4</v></c><c r="F1" s="1" t="s"><v>5</v></c><c r="G1" s="1" t="s"><v>6</v></c><c r="H1" s="1" t="s"><v>7</v></c><c r="I1" s="1" t="s"><v>8</v></c><c r="J1" s="1" t="s"><v>9</v></c><c r="K1" s="1" t="s"><v>10</v></c><c r="L1" s="1" t="s"><v>11</v></c><c r="M1" s="1" t="s"><v>12</v></c><c r="N1" s="1" t="s"><v>13</v></c><c r="O1" s="1" t="s"><v>14</v></c><c r="P1" s="1" t="s"><v>15</v></c><c r="Q1" s="1" t="s"><v>16</v></c><c r="R1" s="1" t="s"><v>17</v></c><c r="S1" s="1" t="s"><v>18</v></c><c r="T1" s="1" t="s"><v>19</v></c><c r="U1" s="1" t="s"><v>20</v></c><c r="V1" s="1" t="s"><v>21</v></c><c r="W1" s="1" t="s"><v>22</v></c><c r="X1" s="1" t="s"><v>23</v></c><c r="Y1" s="1" t="s"><v>24</v></c><c r="Z1" s="1" t="s"><v>25</v></c><c r="AA1" s="1" t="s"><v>26</v></c><c r="AB1" s="1" t="s"><v>27</v></c><c r="AC1" s="1" t="s"><v>28</v></c><c r="AD1" s="1" t="s"><v>29</v></c><c r="AE1" s="1" t="s"><v>30</v></c><c r="AF1" s="1" t="s"><v>31</v></c><c r="AG1" s="1" t="s"><v>32</v></c><c r="AH1" s="1" t="s"><v>33</v></c><c r="AI1" s="1" t="s"><v>34</v></c><c r="AJ1" s="1" t="s"><v>35</v></c><c r="AK1" s="1" t="s"><v>36</v></c><c r="AL1" s="1" t="s"><v>37</v></c><c r="AM1" s="1" t="s"><v>38</v></c></row><row r="2"><c r="A2" s="2" t="s"><v>39</v></c><c r="B2" s="2" t="s"><v>40</v></c><c r="C2" s="2" t="s"><v>41</v></c><c r="D2" s="2" t="s"><v>42</v></c><c r="E2" s="2" t="s"><v>43</v></c><c r="F2" s="2" t="s"><v>44</v></c><c r="G2" s="2" t="s"><v>45</v></c><c r="H2" s="2" t="s"><v>46</v></c><c r="I2" s="2" t="s"><v>47</v></c><c r="J2" s="2" t="s"><v>48</v></c><c r="K2" s="2" t="s"><v>49</v></c><c r="L2" s="2" t="s"><v>50</v></c><c r="M2" s="2" t="s"><v>48</v></c><c r="N2" s="2" t="s"><v>51</v></c><c r="O2" s="2" t="s"><v>52</v></c><c r="P2" s="2" t="s"><v>53</v></c><c r="Q2" s="2" t="s"><v>54</v></c><c r="R2" s="2" t="s"><v>55</v></c><c r="S2" s="2" t="s"><v>56</v></c><c r="T2" s="2" t="s"><v>48</v></c><c r="U2" s="2" t="s"><v>57</v></c><c r="V2" s="2" t="s"><v>48</v></c><c r="W2" s="2" t="s"><v>48</v></c><c r="X2" s="2" t="s"><v>57</v></c><c r="Y2" s="2" t="s"><v>57</v></c><c r="Z2" s="2" t="s"><v>57</v></c><c r="AA2" s="2" t="s"><v>57</v></c><c r="AB2" s="2" t="s"><v>57</v></c><c r="AC2" s="2" t="s"><v>57</v></c><c r="AD2" s="2" t="s"><v>57</v></c><c r="AE2" s="2" t="s"><v>58</v></c><c r="AF2" s="2" t="s"><v>59</v></c><c r="AG2" s="2" t="s"><v>60</v></c><c r="AH2" s="2" t="s"><v>61</v></c><c r="AI2" s="2" t="s"><v>62</v></c><c r="AJ2" s="2" t="s"><v>63</v></c><c r="AK2" s="2" t="s"><v>64</v></c><c r="AL2" s="2" t="s"><v>65</v></c><c r="AM2" s="2" t="s"><v>66</v></c></row></sheetData><dataValidations count="5"><dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N1001"><formula1>0</formula1></dataValidation><dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P1001"><formula1>0</formula1><formula2>14</formula2></dataValidation><dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q1001"><formula1>0</formula1></dataValidation><dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R1001"><formula1>0</formula1></dataValidation><dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S1001"><formula1>-10</formula1><formula2>40</formula2></dataValidation></dataValidations><pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/><pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/><extLst><ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main"><x14:dataValidations count="20" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main"><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"NAD83,WGS84"</xm:f></x14:formula1><xm:sqref>H2:H1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>J2:J1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>M2:M1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"None,Surface,Subsurface,Both"</xm:f></x14:formula1><xm:sqref>O2:O1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>T2:T1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>U2:U1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>V2:V1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>W2:W1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>X2:X1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>Y2:Y1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>Z2:Z1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>AA2:AA1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>AB2:AB1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>AC2:AC1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"TRUE,FALSE"</xm:f></x14:formula1><xm:sqref>AD2:AD1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"Ephemeral < 7 days,Temporary (1 - 4 wk),Seasonal (5-17 wk),Semi-Permanent (18 - 40 wk),Intermittent (41 - 51 wk),Permanent (52 wk)"</xm:f></x14:formula1><xm:sqref>AE2:AE1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"Wetland,Non-wetland,Inconclusive"</xm:f></x14:formula1><xm:sqref>AF2:AF1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"Met,Not met,Marginal"</xm:f></x14:formula1><xm:sqref>AG2:AG1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"1,2,3,4,5,6,7"</xm:f></x14:formula1><xm:sqref>AK2:AK1001</xm:sqref></x14:dataValidation><x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1"><x14:formula1><xm:f>"AK,WMVC,GP,NCNE"</xm:f></x14:formula1><xm:sqref>AL2:AL1001</xm:sqref></x14:dataValidation></x14:dataValidations></ext></extLst></worksheet>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FF2E5090"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="14.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="12.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="16.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="12.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="12.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="9.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="22.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="9.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="12.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="16.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="10.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="10.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="12.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="7.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="8.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="8.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="8.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="10.71" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="10.71" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="10.71" hidden="0" customWidth="1"/>
+    <col min="23" max="23" width="10.71" hidden="0" customWidth="1"/>
+    <col min="24" max="24" width="10.71" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="10.71" hidden="0" customWidth="1"/>
+    <col min="26" max="26" width="10.71" hidden="0" customWidth="1"/>
+    <col min="27" max="27" width="10.71" hidden="0" customWidth="1"/>
+    <col min="28" max="28" width="10.71" hidden="0" customWidth="1"/>
+    <col min="29" max="29" width="10.71" hidden="0" customWidth="1"/>
+    <col min="30" max="30" width="10.71" hidden="0" customWidth="1"/>
+    <col min="31" max="31" width="13.71" hidden="0" customWidth="1"/>
+    <col min="32" max="32" width="11.71" hidden="0" customWidth="1"/>
+    <col min="33" max="33" width="10.71" hidden="0" customWidth="1"/>
+    <col min="34" max="34" width="10.71" hidden="0" customWidth="1"/>
+    <col min="35" max="35" width="10.71" hidden="0" customWidth="1"/>
+    <col min="36" max="36" width="9.71" hidden="0" customWidth="1"/>
+    <col min="37" max="37" width="9.71" hidden="0" customWidth="1"/>
+    <col min="38" max="38" width="40.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AH2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AI2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AJ2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="AK2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="AL2" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N1001">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P1001">
+      <formula1>0</formula1>
+      <formula2>14</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q1001">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R1001">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S1001">
+      <formula1>-10</formula1>
+      <formula2>40</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="19">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"NAD83,WGS84"</xm:f>
+          </x14:formula1>
+          <xm:sqref>H2:H1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>J2:J1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>M2:M1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"None,Surface,Subsurface,Both"</xm:f>
+          </x14:formula1>
+          <xm:sqref>O2:O1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>T2:T1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>U2:U1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>V2:V1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>W2:W1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>X2:X1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>Y2:Y1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>Z2:Z1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>AA2:AA1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>AB2:AB1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>AC2:AC1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>AD2:AD1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Wetland,Non-wetland,Inconclusive"</xm:f>
+          </x14:formula1>
+          <xm:sqref>AE2:AE1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Met,Not met,Marginal"</xm:f>
+          </x14:formula1>
+          <xm:sqref>AF2:AF1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"1,2,3,4,5,6,7"</xm:f>
+          </x14:formula1>
+          <xm:sqref>AJ2:AJ1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"AK,WMVC,GP,NCNE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>AK2:AK1001</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -697,45 +1113,45 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -782,50 +1198,50 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" ht="80" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Drop ecosite columns from vegetation Excel template
ecosite / nm_regime / tree_mod removed from the plots sheet —
matches the recent removal of the Ecosite Classification section
from vegetation_hydrology_field_form.pdf. These attributes will be
assigned in 03_transform.Rmd from external sources rather than
collected on the field form.

structural_stage stays as a numeric 1-7 dropdown so the column
remains friendly for math and downstream filtering; the stage-name
labels (Herb / Shrub / sapling / pole / Young / Mature / Old Forest)
get attached at the transform or visualize stage rather than baked
into the data-entry choices.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/templates/vegetation_hydrology_data_entry.xlsx
+++ b/inst/templates/vegetation_hydrology_data_entry.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
   <si>
     <t xml:space="preserve">project_id</t>
   </si>
@@ -112,15 +112,6 @@
     <t xml:space="preserve">dom_criterion</t>
   </si>
   <si>
-    <t xml:space="preserve">ecosite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nm_regime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tree_mod</t>
-  </si>
-  <si>
     <t xml:space="preserve">structural_stage</t>
   </si>
   <si>
@@ -191,15 +182,6 @@
   </si>
   <si>
     <t xml:space="preserve">Met</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w2b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sw</t>
   </si>
   <si>
     <t xml:space="preserve">3</t>
@@ -706,12 +688,9 @@
     <col min="30" max="30" width="10.71" hidden="0" customWidth="1"/>
     <col min="31" max="31" width="13.71" hidden="0" customWidth="1"/>
     <col min="32" max="32" width="11.71" hidden="0" customWidth="1"/>
-    <col min="33" max="33" width="10.71" hidden="0" customWidth="1"/>
-    <col min="34" max="34" width="10.71" hidden="0" customWidth="1"/>
-    <col min="35" max="35" width="10.71" hidden="0" customWidth="1"/>
-    <col min="36" max="36" width="9.71" hidden="0" customWidth="1"/>
-    <col min="37" max="37" width="9.71" hidden="0" customWidth="1"/>
-    <col min="38" max="38" width="40.71" hidden="0" customWidth="1"/>
+    <col min="33" max="33" width="9.71" hidden="0" customWidth="1"/>
+    <col min="34" max="34" width="9.71" hidden="0" customWidth="1"/>
+    <col min="35" max="35" width="40.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -820,130 +799,112 @@
       <c r="AI1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>37</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="M2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="M2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="N2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="T2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="U2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="V2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="AF2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="T2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="U2" s="2" t="s">
+      <c r="AG2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="V2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="AC2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="AE2" s="2" t="s">
+      <c r="AH2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="AF2" s="2" t="s">
+      <c r="AI2" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="AG2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AH2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI2" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="AJ2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="AK2" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="AL2" s="2" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1077,13 +1038,13 @@
           <x14:formula1>
             <xm:f>"1,2,3,4,5,6,7"</xm:f>
           </x14:formula1>
-          <xm:sqref>AJ2:AJ1001</xm:sqref>
+          <xm:sqref>AG2:AG1001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"AK,WMVC,GP,NCNE"</xm:f>
           </x14:formula1>
-          <xm:sqref>AK2:AK1001</xm:sqref>
+          <xm:sqref>AH2:AH1001</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1113,45 +1074,45 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1198,50 +1159,50 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" ht="80" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Identify species by scientific name, not species code
Replace the field-collected species code with a common name + scientific
name pair on the vegetation/hydrology form, and key all downstream
species resolution on the scientific (Latin) name.

- Excel/PDF templates: species sheet column spp_code -> spp_common
  (Common Name) beside spp_name (Scientific Name); regenerated artifacts.
- 01_ingest: rename spp_common -> common_name, spp_name -> scientific_name;
  drop the species_code rename. common_name is carried as a label only.
- 02_qaqc: unrecognised-species check now matches scientific_name against
  awcs_wetland_species and wetland_indicator_status (excludes non-veg rows);
  required-fields check requires an identity (scientific or common name)
  so bare-ground rows are not dropped.
- 03_transform / 04_visualize: drop species_code references.
- WORKFLOW.md / README.md: wording corrected.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/templates/vegetation_hydrology_data_entry.xlsx
+++ b/inst/templates/vegetation_hydrology_data_entry.xlsx
@@ -193,7 +193,7 @@
     <t xml:space="preserve">Riparian marsh. Saturated at surface throughout.</t>
   </si>
   <si>
-    <t xml:space="preserve">spp_code</t>
+    <t xml:space="preserve">spp_common</t>
   </si>
   <si>
     <t xml:space="preserve">spp_name</t>
@@ -211,7 +211,7 @@
     <t xml:space="preserve">notes</t>
   </si>
   <si>
-    <t xml:space="preserve">TYPH.LATI</t>
+    <t xml:space="preserve">Common cattail</t>
   </si>
   <si>
     <t xml:space="preserve">Typha latifolia</t>
@@ -256,13 +256,13 @@
     <t xml:space="preserve">species — columns</t>
   </si>
   <si>
-    <t xml:space="preserve">plot_id: foreign key matching plots sheet | spp_code: ACIMS-style code (4-letter genus + '.' + 4-letter epithet, e.g. TYPH.LATI for Typha latifolia) — must match the spp_code column in the awcs_wetland_species reference table (data/awcs_wetland_species.rda) | spp_name: scientific name (optional — R looks up from reference table) | stratum: T (tree &gt;10 m) / S (shrub &gt;5 m) / G (ground 1x1 m) | invasive: Y if the field crew flagged a suspected infestation, N otherwise (canonical invasive status is still derived from aisc_invasive_plants in 03_transform.Rmd) | notes: free text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SPECIES CODES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Codes follow the ACIMS (Alberta Centre for Information on Alberta Species) binomial convention: first 4 letters of genus + '.' + first 4 letters of specific epithet, all uppercase (e.g. CARE.AQUA, TYPH.LATI, SALI.EXIG). The complete code list is in the R package reference table: data/awcs_wetland_species.rda (column spp_code). Source plant list: Alberta Wetland Plant List (ACIMS / AEP) — INSERT ACIMS URL HERE (contact Alberta Environment and Protected Areas or search 'ACIMS wetland plant list Alberta').</t>
+    <t xml:space="preserve">plot_id: foreign key matching plots sheet | spp_common: common name (human-readable label; carried through but NOT the join key) | spp_name: scientific (Latin) name — the primary identifier. Must match the scientific_name column in the reference tables (data/awcs_wetland_species.rda, data/wetland_indicator_status.rda); all downstream lookups join on this | stratum: T (tree &gt;10 m) / S (shrub &gt;5 m) / G (ground 1x1 m) | invasive: Y if the field crew flagged a suspected infestation, N otherwise (canonical invasive status is still derived from aisc_invasive_plants in 03_transform.Rmd) | notes: free text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPECIES NAMES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identify each species by its scientific (Latin) name in spp_name — this is the key all reference-table lookups join on. Match the binomial exactly as it appears in the reference list, including author abbreviations where present (e.g. 'Typha latifolia', 'Carex aquatilis Wahlenb.'). spp_common is a free-text common name for readability only and is not used for matching. The complete scientific-name list is in the R package reference table: data/awcs_wetland_species.rda (column scientific_name). Source plant list: Alberta Wetland Plant List (ACIMS / AEP) — INSERT ACIMS URL HERE (contact Alberta Environment and Protected Areas or search 'ACIMS wetland plant list Alberta').</t>
   </si>
 </sst>
 </file>
@@ -1061,7 +1061,7 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="12.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="24.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="28.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="8.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="10.71" hidden="0" customWidth="1"/>

</xml_diff>